<commit_message>
Add updated GLMM scripts, datasets, and colour palette script for model selection
</commit_message>
<xml_diff>
--- a/Analysis/clean data/Formatted for viewing_Survey 1 & 2_scored_near complete_16.6.26.xlsx
+++ b/Analysis/clean data/Formatted for viewing_Survey 1 & 2_scored_near complete_16.6.26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ranidavis/Desktop/Bats &amp; agriculture/Beneficial Bats - collaborative paper/IBRC paper analysis/IBRC beneficial bats survey response analysis/Analysis/clean data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09048272-3F30-154E-9513-10AF5ED772AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A15871-54AF-CE4B-96FD-E3668A05E01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35560" yWindow="-2100" windowWidth="33120" windowHeight="19380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Survey 1 - Knowledge" sheetId="1" r:id="rId1"/>
@@ -17091,10 +17091,10 @@
         <v>771</v>
       </c>
       <c r="E53" s="45" t="s">
-        <v>638</v>
+        <v>467</v>
       </c>
       <c r="F53" s="45" t="s">
-        <v>639</v>
+        <v>100</v>
       </c>
       <c r="G53" t="s">
         <v>101</v>

</xml_diff>